<commit_message>
incomplete updates for new acro codes
</commit_message>
<xml_diff>
--- a/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
+++ b/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leahy\RustroverProjects\check_cards\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD1FBC0-04E1-4942-BA54-8D392483C6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E575671-881D-4CB8-9593-532AE252177A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8987486B-5DC1-406A-92BD-FEEC5C92F2E7}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{8987486B-5DC1-406A-92BD-FEEC5C92F2E7}"/>
   </bookViews>
   <sheets>
     <sheet name="SENIOR-Team_Free-PRELIMS-OCC-" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="66">
   <si>
     <t xml:space="preserve">2024 | COACH CARD    </t>
   </si>
@@ -210,21 +210,6 @@
     <t>3:08-3:14</t>
   </si>
   <si>
-    <t>3:15-3:26</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> AB A6 RB A1c RO1 F2b</t>
-  </si>
-  <si>
-    <t>3PC</t>
-  </si>
-  <si>
-    <t>B3BC</t>
-  </si>
-  <si>
-    <t>3:27-3:29</t>
-  </si>
-  <si>
     <t>Club: ________________________________________________________________</t>
   </si>
   <si>
@@ -240,16 +225,16 @@
     <t>C-Thr^2F-Forw-ow/2ln</t>
   </si>
   <si>
-    <t xml:space="preserve"> A3a A6 A1c A6 F4f*0.3 F4e*0.5 F4f*0.5 F4f A1d</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CB+ A5 1RB A6 CB+ CB+ A1c 2RB</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> FB F6a AB A6 S1 AB 2R1 F1a F2b F3b</t>
-  </si>
-  <si>
     <t>ISS Coach Card Version: 3.0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FB F6a AB A8 S1 AB 2R1 F1a F2b F3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A3a A8 A1c A8 F4f*0.3 F4e*0.5 F4f*0.5 F4f A1d</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CB+ A5 1RB A8 CB+ CB+ A1c 2RB</t>
   </si>
 </sst>
 </file>
@@ -791,19 +776,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1D3D526-A40C-4C69-8373-29C6A2FBDE73}">
-  <dimension ref="A1:H60"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H58"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="10.5546875" customWidth="1"/>
-    <col min="3" max="3" width="6.5546875" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" customWidth="1"/>
-    <col min="5" max="5" width="27.5546875" customWidth="1"/>
-    <col min="6" max="6" width="9.5546875" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
-    <col min="8" max="8" width="6.5546875" customWidth="1"/>
+    <col min="1" max="2" width="10.53125" customWidth="1"/>
+    <col min="3" max="3" width="6.53125" customWidth="1"/>
+    <col min="4" max="4" width="10.53125" customWidth="1"/>
+    <col min="5" max="5" width="27.53125" customWidth="1"/>
+    <col min="6" max="6" width="9.53125" customWidth="1"/>
+    <col min="7" max="7" width="10.53125" customWidth="1"/>
+    <col min="8" max="8" width="6.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -815,7 +800,7 @@
       <c r="G1" s="22"/>
       <c r="H1" s="23"/>
     </row>
-    <row r="2" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
@@ -829,7 +814,7 @@
       <c r="G2" s="18"/>
       <c r="H2" s="19"/>
     </row>
-    <row r="3" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="17" t="s">
         <v>3</v>
       </c>
@@ -841,7 +826,7 @@
       <c r="G3" s="18"/>
       <c r="H3" s="19"/>
     </row>
-    <row r="4" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
@@ -855,21 +840,21 @@
       <c r="G4" s="18"/>
       <c r="H4" s="19"/>
     </row>
-    <row r="5" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A5" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="16"/>
       <c r="D5" s="20" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E5" s="18"/>
       <c r="F5" s="18"/>
       <c r="G5" s="18"/>
       <c r="H5" s="19"/>
     </row>
-    <row r="6" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="17" t="s">
         <v>7</v>
       </c>
@@ -881,7 +866,7 @@
       <c r="G6" s="18"/>
       <c r="H6" s="19"/>
     </row>
-    <row r="7" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="17" t="s">
         <v>8</v>
       </c>
@@ -895,7 +880,7 @@
       <c r="G7" s="18"/>
       <c r="H7" s="19"/>
     </row>
-    <row r="8" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -907,7 +892,7 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
     </row>
-    <row r="9" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="13" t="s">
         <v>11</v>
       </c>
@@ -919,7 +904,7 @@
       <c r="G9" s="14"/>
       <c r="H9" s="15"/>
     </row>
-    <row r="10" spans="1:8" ht="29.4" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="28.9" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
@@ -945,7 +930,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
@@ -959,7 +944,7 @@
       <c r="G11" s="8"/>
       <c r="H11" s="9"/>
     </row>
-    <row r="12" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A12" s="7" t="s">
         <v>22</v>
       </c>
@@ -983,7 +968,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A13" s="7" t="s">
         <v>27</v>
       </c>
@@ -997,7 +982,7 @@
       <c r="G13" s="8"/>
       <c r="H13" s="9"/>
     </row>
-    <row r="14" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="7" t="s">
         <v>28</v>
       </c>
@@ -1011,7 +996,7 @@
         <v>29</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="8">
@@ -1021,7 +1006,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A15" s="7" t="s">
         <v>31</v>
       </c>
@@ -1035,7 +1020,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="9"/>
     </row>
-    <row r="16" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A16" s="7" t="s">
         <v>32</v>
       </c>
@@ -1059,7 +1044,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A17" s="7" t="s">
         <v>36</v>
       </c>
@@ -1073,7 +1058,7 @@
       <c r="G17" s="8"/>
       <c r="H17" s="9"/>
     </row>
-    <row r="18" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A18" s="7" t="s">
         <v>37</v>
       </c>
@@ -1085,19 +1070,19 @@
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="11" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>39</v>
       </c>
       <c r="G18" s="8">
-        <v>4.05</v>
+        <v>3.9</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A19" s="7" t="s">
         <v>41</v>
       </c>
@@ -1111,7 +1096,7 @@
       <c r="G19" s="8"/>
       <c r="H19" s="9"/>
     </row>
-    <row r="20" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="7" t="s">
         <v>42</v>
       </c>
@@ -1123,19 +1108,19 @@
       </c>
       <c r="D20" s="7"/>
       <c r="E20" s="12" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G20" s="8">
-        <v>4.92</v>
+        <v>4.8049999999999997</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="7" t="s">
         <v>45</v>
       </c>
@@ -1149,7 +1134,7 @@
       <c r="G21" s="8"/>
       <c r="H21" s="9"/>
     </row>
-    <row r="22" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="7" t="s">
         <v>46</v>
       </c>
@@ -1161,19 +1146,19 @@
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="6" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G22" s="8">
-        <v>3.8</v>
+        <v>3.85</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="7" t="s">
         <v>49</v>
       </c>
@@ -1187,7 +1172,7 @@
       <c r="G23" s="8"/>
       <c r="H23" s="9"/>
     </row>
-    <row r="24" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A24" s="7" t="s">
         <v>50</v>
       </c>
@@ -1199,7 +1184,7 @@
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="11" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>39</v>
@@ -1211,7 +1196,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A25" s="7" t="s">
         <v>52</v>
       </c>
@@ -1225,7 +1210,7 @@
       <c r="G25" s="8"/>
       <c r="H25" s="9"/>
     </row>
-    <row r="26" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A26" s="7" t="s">
         <v>53</v>
       </c>
@@ -1241,13 +1226,13 @@
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="8">
-        <v>2.5499999999999998</v>
+        <v>2.7</v>
       </c>
       <c r="H26" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A27" s="7" t="s">
         <v>56</v>
       </c>
@@ -1261,34 +1246,18 @@
       <c r="G27" s="8"/>
       <c r="H27" s="9"/>
     </row>
-    <row r="28" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="7">
-        <v>9</v>
-      </c>
+    <row r="28" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A28" s="7"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="7"/>
       <c r="D28" s="7"/>
-      <c r="E28" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G28" s="8">
-        <v>3.25</v>
-      </c>
-      <c r="H28" s="10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="7" t="s">
-        <v>61</v>
-      </c>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="9"/>
+    </row>
+    <row r="29" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A29" s="7"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
@@ -1297,7 +1266,7 @@
       <c r="G29" s="8"/>
       <c r="H29" s="9"/>
     </row>
-    <row r="30" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="7"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7"/>
@@ -1307,7 +1276,7 @@
       <c r="G30" s="8"/>
       <c r="H30" s="9"/>
     </row>
-    <row r="31" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A31" s="7"/>
       <c r="B31" s="6"/>
       <c r="C31" s="7"/>
@@ -1317,7 +1286,7 @@
       <c r="G31" s="8"/>
       <c r="H31" s="9"/>
     </row>
-    <row r="32" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A32" s="7"/>
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
@@ -1327,7 +1296,7 @@
       <c r="G32" s="8"/>
       <c r="H32" s="9"/>
     </row>
-    <row r="33" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A33" s="7"/>
       <c r="B33" s="6"/>
       <c r="C33" s="7"/>
@@ -1337,28 +1306,32 @@
       <c r="G33" s="8"/>
       <c r="H33" s="9"/>
     </row>
-    <row r="34" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="7"/>
-      <c r="B34" s="6"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="9"/>
-    </row>
-    <row r="35" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="9"/>
-    </row>
-    <row r="36" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="1"/>
+    <row r="34" spans="1:8" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A35" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A36" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1367,7 +1340,7 @@
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
         <v>62</v>
       </c>
@@ -1379,10 +1352,8 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>63</v>
-      </c>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
@@ -1391,10 +1362,8 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>70</v>
-      </c>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
@@ -1403,7 +1372,7 @@
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1413,7 +1382,7 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1423,7 +1392,7 @@
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
@@ -1433,7 +1402,7 @@
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1443,7 +1412,7 @@
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
@@ -1453,7 +1422,7 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
@@ -1463,7 +1432,7 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1473,7 +1442,7 @@
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
@@ -1483,7 +1452,7 @@
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
@@ -1493,7 +1462,7 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
@@ -1503,7 +1472,7 @@
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
@@ -1513,7 +1482,7 @@
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
@@ -1523,7 +1492,7 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
@@ -1533,7 +1502,7 @@
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -1543,7 +1512,7 @@
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
@@ -1553,7 +1522,7 @@
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
@@ -1563,7 +1532,7 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
@@ -1573,7 +1542,7 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
@@ -1583,7 +1552,7 @@
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
@@ -1592,26 +1561,6 @@
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
more updates for the new changes
</commit_message>
<xml_diff>
--- a/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
+++ b/tests/SENIOR-Team_Free-PRELIMS-OCC-.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leahy\RustroverProjects\check_cards\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E575671-881D-4CB8-9593-532AE252177A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A9A3AAC-83E2-4833-822B-CAC21DA17FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{8987486B-5DC1-406A-92BD-FEEC5C92F2E7}"/>
   </bookViews>
@@ -201,9 +201,6 @@
     <t>2:50-3:07</t>
   </si>
   <si>
-    <t xml:space="preserve"> T3d A2b A2b A2b A3a S2</t>
-  </si>
-  <si>
     <t>7589</t>
   </si>
   <si>
@@ -219,9 +216,6 @@
     <t>Test</t>
   </si>
   <si>
-    <t xml:space="preserve"> C4 C4 C4 RD2 S1</t>
-  </si>
-  <si>
     <t>C-Thr^2F-Forw-ow/2ln</t>
   </si>
   <si>
@@ -234,7 +228,13 @@
     <t xml:space="preserve"> A3a A8 A1c A8 F4f*0.3 F4e*0.5 F4f*0.5 F4f A1d</t>
   </si>
   <si>
-    <t xml:space="preserve"> CB+ A5 1RB A8 CB+ CB+ A1c 2RB</t>
+    <t xml:space="preserve"> C4 C4 RD2 S1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CB+ A5 1RB A8 CB+ A1c 2RB</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> T3d A2b A2b A3a S2</t>
   </si>
 </sst>
 </file>
@@ -419,16 +419,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -442,6 +432,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,96 +789,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="45" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="23"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="20" t="s">
+      <c r="B2" s="14"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="19"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="15"/>
     </row>
     <row r="3" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="19"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="15"/>
     </row>
     <row r="4" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="20" t="s">
+      <c r="B4" s="14"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="19"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="19"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="20" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="19"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="2" t="s">
@@ -893,16 +893,16 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="15"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="22"/>
     </row>
     <row r="10" spans="1:8" ht="28.9" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="3" t="s">
@@ -996,7 +996,7 @@
         <v>29</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="8">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>39</v>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="D20" s="7"/>
       <c r="E20" s="12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>43</v>
@@ -1146,13 +1146,13 @@
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G22" s="8">
-        <v>3.85</v>
+        <v>3.35</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>48</v>
@@ -1184,13 +1184,13 @@
       </c>
       <c r="D24" s="7"/>
       <c r="E24" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>39</v>
       </c>
       <c r="G24" s="8">
-        <v>3.55</v>
+        <v>3.35</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>51</v>
@@ -1222,19 +1222,19 @@
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="6" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="8">
-        <v>2.7</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A27" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>21</v>
@@ -1318,7 +1318,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -1330,7 +1330,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1342,7 +1342,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A37" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -1564,6 +1564,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:H7"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="D4:H4"/>
     <mergeCell ref="A1:H1"/>
@@ -1571,13 +1578,6 @@
     <mergeCell ref="D2:H2"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="D3:H3"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:H7"/>
   </mergeCells>
   <pageMargins left="6.9444444444444441E-3" right="6.9444444444444441E-3" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>